<commit_message>
Postergación de tareas por cuello de botella (con motivo)
- Nueva hoja "Postergar": por cada tarea, dos listas desplegables
  -> "Postergar (nº sprints)" (0-3; 1 = próximo) y "Motivo del cuello de
  botella" (lista editable: dependencia, sobrecarga, falta de info,
  reestimación, recurso, prioridad, bloqueo técnico, otro).
- Sprint vigente = MÁX(planificado, sprint actual) + postergación manual;
  el movimiento y su motivo quedan en "Historial de Sprints" (auto).
- Botón opcional de 1 clic: macro PostergarTareaActual (macro_sprints.bas)
  rellena esas celdas y elige el motivo por lista.
- Validación de datos (listas) + resaltado de celdas editables.
- Guía y README actualizados. Hoja Gantt y hojas originales intactas.

https://claude.ai/code/session_01T2X5Sdkmy5GoJRwojb8uhJ
</commit_message>
<xml_diff>
--- a/Guia_Diagrama_de_Gantt.xlsx
+++ b/Guia_Diagrama_de_Gantt.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I34"/>
+  <dimension ref="B1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -612,122 +612,130 @@
       <c r="H21" s="5" t="n"/>
       <c r="I21" s="5" t="n"/>
     </row>
-    <row r="22" ht="50" customHeight="1">
+    <row r="22" ht="46" customHeight="1">
       <c r="B22" s="3" t="inlineStr">
         <is>
           <t>En 'Historial de Sprints' se define Inicio Sprint 1 y Duración (editables). Sprint actual = ENTERO((HOY−Inicio)/Duración)+1. Regla: si una tarea NO está 'Completada' y su sprint ya cerró, su 'Sprint vigente' = sprint actual (se reasigna automáticamente al siguiente). El Sprint planificado original (col E del Gantt) NO se toca: queda como histórico. Todo es por fórmula, se recalcula solo al abrir/cambiar fechas.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="4" t="inlineStr">
+    <row r="23" ht="46" customHeight="1">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Postergar manual por cuello de botella (hoja 'Postergar'): en la fila de la tarea elija 'Postergar (nº sprints)' (lista 0-3; 1 = próximo) y el 'Motivo' (lista editable: dependencia, sobrecarga, falta de info, reestimación, recurso, prioridad, bloqueo técnico, otro). El Sprint vigente se ajusta solo y el movimiento queda registrado con ese motivo. Botón opcional de 1 clic: macro 'PostergarTareaActual' (archivo macro_sprints.bas) — asígnela a un botón de formulario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>4) TRAZABILIDAD (Historial de Sprints)</t>
         </is>
       </c>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
-    </row>
-    <row r="25" ht="34" customHeight="1">
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Registra cada reasignación: ID de tarea, Tarea, Responsable, Sprint origen, Sprint destino, Fecha del movimiento (cierre del sprint origen) y Motivo. Se completa automáticamente con las tareas cuyo Sprint vigente ≠ Sprint planificado.</t>
-        </is>
-      </c>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="n"/>
+      <c r="I25" s="5" t="n"/>
     </row>
     <row r="26" ht="34" customHeight="1">
       <c r="B26" s="3" t="inlineStr">
         <is>
+          <t>Registra cada reasignación: ID de tarea, Tarea, Responsable, Sprint origen, Sprint destino, Fecha del movimiento (cierre del sprint origen) y Motivo. Se completa automáticamente con las tareas cuyo Sprint vigente ≠ Sprint planificado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
           <t>Para un registro PERSISTENTE con write-back físico + usuario de Windows, use la macro opcional 'macro_sprints.bas' (ver README): reasigna el nº de sprint en el Gantt y agrega una línea con fecha/usuario. Requiere guardar como .xlsm.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="4" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>ESCALABILIDAD</t>
         </is>
       </c>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="B29" s="3" t="inlineStr">
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="5" t="n"/>
+      <c r="I29" s="5" t="n"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Las fórmulas llegan a la fila 200 del Gantt. Para superar 200 filas, amplíe el rango en _Datos. Los sprints aparecen solos al usarse (lista dinámica) y conservan el histórico.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="4" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>OBSERVACIONES (no se modificaron datos; se informan para revisión)</t>
         </is>
       </c>
-      <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
-    </row>
-    <row r="32" ht="40" customHeight="1">
-      <c r="B32" s="3" t="inlineStr">
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
+      <c r="I32" s="5" t="n"/>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>• Promedios de fase J27 y J36: promedian rangos que no corresponden (38% y 17% cuando el real es 72% y 43%). El Tablero ya lo recalcula bien. Para corregir el origen: J27 → =PROMEDIO(J28:J35) ; J36 → =PROMEDIO(J37:J47).</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="B33" s="3" t="inlineStr">
+    <row r="34" ht="30" customHeight="1">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>• Fechas a revisar: K13 (19/11/2026, posterior al FIN), K40 (01/12/2026) y filas con INICIO &gt; FIN (41,42,46,47) → días negativos.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="3" t="inlineStr">
+    <row r="35" ht="22" customHeight="1">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>• Filas 79-80: textos sueltos sin fecha; se excluyen automáticamente.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="27">
     <mergeCell ref="B7:I7"/>
     <mergeCell ref="B25:I25"/>
     <mergeCell ref="B16:I16"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B22:I22"/>
-    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B27:I27"/>
     <mergeCell ref="B12:I12"/>
     <mergeCell ref="B18:I18"/>
     <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B23:I23"/>
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="B8:I8"/>
     <mergeCell ref="B17:I17"/>
     <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B35:I35"/>
     <mergeCell ref="B29:I29"/>
     <mergeCell ref="B34:I34"/>
     <mergeCell ref="B10:I10"/>
-    <mergeCell ref="B28:I28"/>
     <mergeCell ref="B19:I19"/>
     <mergeCell ref="B9:I9"/>
+    <mergeCell ref="B30:I30"/>
     <mergeCell ref="B15:I15"/>
     <mergeCell ref="B33:I33"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B24:I24"/>
     <mergeCell ref="B5:I5"/>
     <mergeCell ref="B32:I32"/>
     <mergeCell ref="B26:I26"/>

</xml_diff>

<commit_message>
Sprints más simple y prolijo: calendario adaptado, 'pasar al siguiente' y comentario libre
- Calendario adaptado a las reuniones reales del Gantt (semanal, cierres
  martes desde 16/06; editable). Sprint actual = primer sprint cuya
  reunión aún no pasó.
- Hoja "Sprints" más prolija: tareas AGRUPADAS POR MÓDULO (encabezados),
  columnas claras y guía de uso en 3 pasos.
- "Pasar al siguiente": lista Sí (1 clic) para empujar una tarea al
  sprint siguiente, además del paso automático al cerrar la reunión.
- Motivo del desvío: validación de datos (lista editable) +
  COMENTARIO (texto libre, totalmente editable y personalizable).
- _Datos: Sprint vigente = MÁX(planif, actual) + (Pasar="Sí").
- macro_sprints.bas: botones PasarAlSiguiente / IndicarMotivo.
- Guía y README actualizados. Gantt y hojas originales intactos.

https://claude.ai/code/session_01T2X5Sdkmy5GoJRwojb8uhJ
</commit_message>
<xml_diff>
--- a/Guia_Diagrama_de_Gantt.xlsx
+++ b/Guia_Diagrama_de_Gantt.xlsx
@@ -615,28 +615,28 @@
     <row r="22" ht="40" customHeight="1">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Un sprint NO es una tarea: es un PERÍODO de tiempo que cierra en una reunión. En la hoja 'Sprints' hay un CALENDARIO editable (Sprint 1, 2, 3... con su fecha de cierre = la reunión). 'Sprint actual' se calcula solo: es el primer sprint cuya reunión todavía no pasó.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="40" customHeight="1">
+          <t>Un sprint NO es una tarea: es un PERÍODO de tiempo que cierra en una REUNIÓN. En la hoja 'Sprints' hay un CALENDARIO editable (Sprint 1, 2, 3... con la fecha de su reunión de cierre). 'Sprint actual' se calcula solo: es el primer sprint cuya reunión todavía no pasó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Regla (igual que Scrum): al cerrar la reunión de un sprint, las tareas 'Completadas' quedan registradas en ese sprint; las NO completadas pasan automáticamente al sprint siguiente (Sprint vigente), mostrando el DESVÍO en días. El Sprint planificado (col E del Gantt) NO se toca: es el histórico.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="40" customHeight="1">
+          <t>Regla (igual que Scrum): al cerrar la reunión, las tareas 'Completadas' quedan en su sprint; las NO completadas pasan automáticamente al sprint siguiente (Sprint vigente), mostrando el DESVÍO en días. El Sprint planificado (col E del Gantt) NO se toca: es el histórico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Indicar el motivo (cuello de botella): en 'Sprints', columna 'Motivo del desvío', elija de la lista editable (dependencia, sobrecarga, falta de info, reestimación, recurso, prioridad, bloqueo técnico, otro). Es lo único que hay que completar. Botón opcional de 1 clic: macro 'IndicarMotivo' (macro_sprints.bas).</t>
+          <t>Cómo usar la hoja 'Sprints' (3 pasos): 1) edite la fecha de cierre de cada reunión en el calendario; 2) para pasar una tarea al sprint siguiente, elija 'Sí' en la columna 'Pasar al siguiente'; 3) indique el 'Motivo del desvío' (lista editable) y/o escriba un 'Comentario' libre (texto totalmente personalizable). Las filas de cada módulo se agrupan con un encabezado.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>4) TRAZABILIDAD (hoja Sprints)</t>
+          <t>4) TRAZABILIDAD Y MOTIVOS (hoja Sprints)</t>
         </is>
       </c>
       <c r="C26" s="5" t="n"/>
@@ -647,10 +647,10 @@
       <c r="H26" s="5" t="n"/>
       <c r="I26" s="5" t="n"/>
     </row>
-    <row r="27" ht="40" customHeight="1">
+    <row r="27" ht="46" customHeight="1">
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>La tabla 'Seguimiento de tareas por sprint' muestra, por tarea: Sprint planificado → Sprint vigente, el desvío en días y el motivo. Las tareas movidas se resaltan. Para una bitácora PERSISTENTE con fecha/hora y usuario, use la macro opcional 'ReasignarSprintsFisico' (.xlsm) que además reasigna el nº de sprint en el Gantt.</t>
+          <t>La tabla 'Seguimiento de tareas por sprint' muestra por tarea: Sprint planificado → Sprint vigente, el desvío en días, el Motivo (lista) y el Comentario (libre). Las tareas movidas se resaltan en ámbar. Motivo = validación de datos (lista editable en P5:P12); Comentario = texto libre. Botones opcionales (.xlsm): 'PasarAlSiguiente' e 'IndicarMotivo'; y 'ReasignarSprintsFisico' para write-back físico + bitácora con fecha/usuario.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Forecast dentro de Tableros (25%), comentarios del Gantt, historial y Nuevo por sprint
- "Tablero Forecast" reubicado DENTRO del bloque de Tableros (filas 48-51,
  dentro del merge H22:H51 del 25%): ya no figura aparte. El total general
  del OKR sigue siendo 100% (Forecast no suma peso propio). Se desplazaron
  módulos 6 y 7 (a filas 52 y 56) ajustando fórmulas, merges y SUBTOTAL.
- Backlog General: trae el "Comentario (Gantt)" de la 1ª hoja + columna
  "Justificación / Comentario" libre -> registro claro de qué no se hizo y
  por qué (aunque esté justificado). Estado/Acción con color.
- Frecuencias editables por validación de datos (Frecuencia por Proyecto).
- "Nuevo" editable: columna "Sol. en Sprint" indica el sprint de la
  solicitud; "Nuevo S#" solo mientras el sprint actual de su frecuencia
  coincide (nuevo en S1 deja de serlo en S2).
- Datos del Gantt (filas 1-47) intactos; hojas originales 2/3/4 idénticas.

https://claude.ai/code/session_01T2X5Sdkmy5GoJRwojb8uhJ
</commit_message>
<xml_diff>
--- a/Guia_Diagrama_de_Gantt.xlsx
+++ b/Guia_Diagrama_de_Gantt.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I35"/>
+  <dimension ref="B1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -629,7 +629,7 @@
     <row r="25">
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>4) BACKLOG: COMPLETAR / NO REALIZAR / POSTERGAR</t>
+          <t>4) BACKLOG: COMPLETAR / NO REALIZAR + HISTORIAL</t>
         </is>
       </c>
       <c r="C25" s="5" t="n"/>
@@ -640,83 +640,91 @@
       <c r="H25" s="5" t="n"/>
       <c r="I25" s="5" t="n"/>
     </row>
-    <row r="26" ht="44" customHeight="1">
+    <row r="26" ht="46" customHeight="1">
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>En 'Backlog General', por cada subtarea: Estado = 'Completo' o 'No se realizó'. Si NO se realizó, elija la Acción: 'Pasa al siguiente' (va al sprint siguiente y aparece ahí con la misma lógica), 'Baja prioridad' (sigue PENDIENTE pero DEJA de contar días de mora) o 'Cancelado'. El 'Comentario' es texto libre. Las tareas con inicio en la semana actual se marcan 'Nuevo'.</t>
+          <t>En 'Backlog General', por subtarea: Estado = 'Completo' o 'No se realizó'. Si NO se realizó, Acción: 'Pasa al siguiente' (va al sprint siguiente con la misma lógica), 'Baja prioridad' (sigue PENDIENTE pero DEJA de contar días de mora) o 'Cancelado'. Queda el registro de qué no se hizo y por qué: 'Comentario (Gantt)' trae las notas de la 1ª hoja (Gantt) y 'Justificación' es texto libre.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1">
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>El proyecto 'Tablero Forecast' (subtareas: armado de procedimiento; slicer % de incremento sobre venta según factores; factores de clientes con % de incremento) se agregó como solicitud NUEVA de la semana, con la misma clasificación que 'Tablero BI OPEX' (Semanal).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="4" t="inlineStr">
+          <t>Frecuencia por proyecto: editable por lista (validación de datos) en la hoja Sprints. 'Nuevo': se indica el sprint en que se solicitó (columna 'Sol. en Sprint'); deja de figurar como nuevo al avanzar de sprint (ej.: nuevo en S1 -&gt; ya no en S2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>El proyecto 'Tablero Forecast' (subtareas: armado de procedimiento; slicer % de incremento s/venta según factores; factores de clientes con % de incremento) se agregó DENTRO del bloque de Tableros (25% del OKR), no aparte; el total general sigue siendo 100%. Solicitud nueva de la semana, clasificada como 'Tablero BI OPEX' (Semanal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>ESCALABILIDAD</t>
         </is>
       </c>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="n"/>
-      <c r="I29" s="5" t="n"/>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="B30" s="3" t="inlineStr">
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="5" t="n"/>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Las fórmulas llegan a la fila 200 del Gantt. Para superar 200 filas, amplíe el rango en _Datos. El calendario admite hasta 8 sprints (ampliable). Los sprints aparecen solos al usarse y conservan el histórico.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>OBSERVACIONES (no se modificaron datos; se informan para revisión)</t>
         </is>
       </c>
-      <c r="C32" s="5" t="n"/>
-      <c r="D32" s="5" t="n"/>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="5" t="n"/>
-      <c r="I32" s="5" t="n"/>
-    </row>
-    <row r="33" ht="40" customHeight="1">
-      <c r="B33" s="3" t="inlineStr">
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="5" t="n"/>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>• Promedios de fase J27 y J36: promedian rangos que no corresponden (38% y 17% cuando el real es 72% y 43%). El Tablero ya lo recalcula bien. Para corregir el origen: J27 → =PROMEDIO(J28:J35) ; J36 → =PROMEDIO(J37:J47).</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="B34" s="3" t="inlineStr">
+    <row r="35" ht="30" customHeight="1">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>• Fechas a revisar: K13 (19/11/2026, posterior al FIN), K40 (01/12/2026) y filas con INICIO &gt; FIN (41,42,46,47) → días negativos.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1">
-      <c r="B35" s="3" t="inlineStr">
+    <row r="36" ht="22" customHeight="1">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>• Filas 79-80: textos sueltos sin fecha; se excluyen automáticamente.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="B7:I7"/>
     <mergeCell ref="B25:I25"/>
     <mergeCell ref="B16:I16"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B22:I22"/>
+    <mergeCell ref="B31:I31"/>
     <mergeCell ref="B27:I27"/>
     <mergeCell ref="B12:I12"/>
     <mergeCell ref="B18:I18"/>
@@ -726,10 +734,9 @@
     <mergeCell ref="B8:I8"/>
     <mergeCell ref="B17:I17"/>
     <mergeCell ref="B13:I13"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="B29:I29"/>
     <mergeCell ref="B34:I34"/>
     <mergeCell ref="B10:I10"/>
+    <mergeCell ref="B28:I28"/>
     <mergeCell ref="B19:I19"/>
     <mergeCell ref="B9:I9"/>
     <mergeCell ref="B30:I30"/>
@@ -737,7 +744,8 @@
     <mergeCell ref="B33:I33"/>
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B5:I5"/>
-    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B35:I35"/>
     <mergeCell ref="B26:I26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>